<commit_message>
Changed constraint C5 to work on crop_group level instead of crop, need to fix crop allocation function accordingly...
</commit_message>
<xml_diff>
--- a/data/relation_tables.xlsx
+++ b/data/relation_tables.xlsx
@@ -1588,7 +1588,7 @@
         <v>73</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D32" s="1" t="s">
         <v>75</v>
@@ -1608,7 +1608,7 @@
         <v>73</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>75</v>
@@ -1628,7 +1628,7 @@
         <v>73</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>75</v>
@@ -1648,7 +1648,7 @@
         <v>77</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D35" s="1" t="s">
         <v>75</v>

</xml_diff>

<commit_message>
Updated default data from Hannas work
</commit_message>
<xml_diff>
--- a/data/relation_tables.xlsx
+++ b/data/relation_tables.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="204">
   <si>
     <t>CPC</t>
   </si>
@@ -615,6 +615,24 @@
   </si>
   <si>
     <t>Sweet lupin</t>
+  </si>
+  <si>
+    <t>Grey pea</t>
+  </si>
+  <si>
+    <t>Sunflower seeds</t>
+  </si>
+  <si>
+    <t>Lentils, dry</t>
+  </si>
+  <si>
+    <t>Hazelnuts</t>
+  </si>
+  <si>
+    <t>Nut trees</t>
+  </si>
+  <si>
+    <t>Walnuts</t>
   </si>
 </sst>
 </file>
@@ -639,7 +657,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="7"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -665,11 +682,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -950,7 +968,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.140625" bestFit="1" customWidth="1"/>
@@ -2137,6 +2155,106 @@
         <v>192</v>
       </c>
       <c r="F59" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D60" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="E60" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F60" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D61" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="E61" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="F61" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D62" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="E62" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="F62" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="E63" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="F63" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="D64" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="E64" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="F64" s="3" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Work on by-products and conversion factors
</commit_message>
<xml_diff>
--- a/data/relation_tables.xlsx
+++ b/data/relation_tables.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="616" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="634" uniqueCount="231">
   <si>
     <t>CPC</t>
   </si>
@@ -645,42 +645,12 @@
     <t>buttermilk</t>
   </si>
   <si>
-    <t>cattle butcher fat</t>
-  </si>
-  <si>
-    <t>cattle skins</t>
-  </si>
-  <si>
-    <t>cattle slaughterhouse fat</t>
-  </si>
-  <si>
     <t>edible offals</t>
   </si>
   <si>
-    <t>pig butcher fat</t>
-  </si>
-  <si>
-    <t>pig skins</t>
-  </si>
-  <si>
-    <t>pig slaughterhouse fat</t>
-  </si>
-  <si>
     <t>rapeseed cake</t>
   </si>
   <si>
-    <t>sheep offals</t>
-  </si>
-  <si>
-    <t>sheep skins</t>
-  </si>
-  <si>
-    <t>sheep slaughterhouse fat</t>
-  </si>
-  <si>
-    <t>wheat gluten?</t>
-  </si>
-  <si>
     <t>by_prod_group</t>
   </si>
   <si>
@@ -694,6 +664,57 @@
   </si>
   <si>
     <t>slaughterhouse by-products</t>
+  </si>
+  <si>
+    <t>milling by-products from wheat, barley or rye</t>
+  </si>
+  <si>
+    <t>milling by-products from oats</t>
+  </si>
+  <si>
+    <t>slaughterhouse fat</t>
+  </si>
+  <si>
+    <t>skins</t>
+  </si>
+  <si>
+    <t>edible blood</t>
+  </si>
+  <si>
+    <t>butcher fat</t>
+  </si>
+  <si>
+    <t>inedible blood</t>
+  </si>
+  <si>
+    <t>feathers</t>
+  </si>
+  <si>
+    <t>inedible offals</t>
+  </si>
+  <si>
+    <t>barley malt culms</t>
+  </si>
+  <si>
+    <t>pea starch</t>
+  </si>
+  <si>
+    <t>wheat starch</t>
+  </si>
+  <si>
+    <t>wheat oil</t>
+  </si>
+  <si>
+    <t>oat fibers</t>
+  </si>
+  <si>
+    <t>broad bean okara</t>
+  </si>
+  <si>
+    <t>wheat distillers grain</t>
+  </si>
+  <si>
+    <t>wheat gluten</t>
   </si>
 </sst>
 </file>
@@ -3539,182 +3560,260 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>204</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="B2" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="B3" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>219</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>205</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="B6" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="B7" t="s">
+        <v>211</v>
+      </c>
+      <c r="C7" s="1"/>
+    </row>
+    <row r="8" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="C8"/>
+      <c r="D8"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>177</v>
-      </c>
-      <c r="B3" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>206</v>
-      </c>
-      <c r="B4" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>207</v>
-      </c>
-      <c r="B5" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="B12" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>209</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="B19" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="B26" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B30" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>212</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>213</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>183</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>182</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>214</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>215</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>216</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>217</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>178</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>179</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>218</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>180</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>221</v>
-      </c>
     </row>
   </sheetData>
+  <sortState ref="D2:D71">
+    <sortCondition ref="D71"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Data update from Hanna
</commit_message>
<xml_diff>
--- a/data/relation_tables.xlsx
+++ b/data/relation_tables.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="crop" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="644" uniqueCount="234">
   <si>
     <t>CPC</t>
   </si>
@@ -718,6 +718,12 @@
   </si>
   <si>
     <t>Buckwheat</t>
+  </si>
+  <si>
+    <t>hazelnut shells</t>
+  </si>
+  <si>
+    <t>walnut shells</t>
   </si>
 </sst>
 </file>
@@ -3583,7 +3589,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
@@ -3833,6 +3839,22 @@
         <v>211</v>
       </c>
     </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>232</v>
+      </c>
+      <c r="B31" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>233</v>
+      </c>
+      <c r="B32" t="s">
+        <v>212</v>
+      </c>
+    </row>
   </sheetData>
   <sortState ref="D2:D71">
     <sortCondition ref="D71"/>

</xml_diff>

<commit_message>
Added rel for remaining animals
</commit_message>
<xml_diff>
--- a/data/relation_tables.xlsx
+++ b/data/relation_tables.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="677" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="719" uniqueCount="275">
   <si>
     <t>CPC</t>
   </si>
@@ -770,6 +770,84 @@
   </si>
   <si>
     <t>bulls and steers</t>
+  </si>
+  <si>
+    <t>ewes</t>
+  </si>
+  <si>
+    <t>rams</t>
+  </si>
+  <si>
+    <t>lambs</t>
+  </si>
+  <si>
+    <t>low-performing horses</t>
+  </si>
+  <si>
+    <t>medium-performing horses</t>
+  </si>
+  <si>
+    <t>broodmares</t>
+  </si>
+  <si>
+    <t>young horses</t>
+  </si>
+  <si>
+    <t>sows</t>
+  </si>
+  <si>
+    <t>boars</t>
+  </si>
+  <si>
+    <t>piglets</t>
+  </si>
+  <si>
+    <t>gilts</t>
+  </si>
+  <si>
+    <t>growing pigs</t>
+  </si>
+  <si>
+    <t>finishing pigs</t>
+  </si>
+  <si>
+    <t>broilers</t>
+  </si>
+  <si>
+    <t>breeding hens</t>
+  </si>
+  <si>
+    <t>breeding roosters</t>
+  </si>
+  <si>
+    <t>laying chicks</t>
+  </si>
+  <si>
+    <t>laying hens (16-28 weeks)</t>
+  </si>
+  <si>
+    <t>laying hens (29-59 weeks)</t>
+  </si>
+  <si>
+    <t>laying hens (&gt;59 weeks)</t>
+  </si>
+  <si>
+    <t>breeding hens and roosters</t>
+  </si>
+  <si>
+    <t>sheep</t>
+  </si>
+  <si>
+    <t>horses</t>
+  </si>
+  <si>
+    <t>other pigs</t>
+  </si>
+  <si>
+    <t>pigs for meat</t>
+  </si>
+  <si>
+    <t>other poultry</t>
   </si>
 </sst>
 </file>
@@ -799,12 +877,30 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -819,13 +915,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2424,133 +2524,322 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="5" t="s">
         <v>234</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="5" t="s">
         <v>246</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="5" t="s">
         <v>247</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="6" t="s">
         <v>236</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="6" t="s">
         <v>236</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="6" t="s">
         <v>236</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="A3" s="6" t="s">
         <v>237</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="6" t="s">
         <v>237</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="6" t="s">
         <v>248</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="7" t="s">
         <v>241</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="7" t="s">
         <v>241</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="6" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="7" t="s">
         <v>242</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="6" t="s">
         <v>240</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="6" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="A6" s="6" t="s">
         <v>243</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="6" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="A7" s="6" t="s">
         <v>244</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="6" t="s">
         <v>239</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="6" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="A8" s="6" t="s">
         <v>245</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="6" t="s">
         <v>240</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="6" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="7" t="s">
         <v>238</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="A10" s="6" t="s">
         <v>239</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="6" t="s">
         <v>239</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="6" t="s">
         <v>248</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="A11" s="6" t="s">
         <v>240</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="6" t="s">
         <v>240</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" s="6" t="s">
         <v>248</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="B12" s="8"/>
+      <c r="C12" s="8" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="B13" s="8"/>
+      <c r="C13" s="8" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="8" t="s">
+        <v>251</v>
+      </c>
+      <c r="B14" s="8"/>
+      <c r="C14" s="8" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
+        <v>252</v>
+      </c>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="9" t="s">
+        <v>256</v>
+      </c>
+      <c r="B19" s="8"/>
+      <c r="C19" s="8" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="B20" s="8"/>
+      <c r="C20" s="8" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="B21" s="8"/>
+      <c r="C21" s="8" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="8" t="s">
+        <v>259</v>
+      </c>
+      <c r="B22" s="8"/>
+      <c r="C22" s="8" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="8" t="s">
+        <v>260</v>
+      </c>
+      <c r="B23" s="8"/>
+      <c r="C23" s="8" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="8" t="s">
+        <v>261</v>
+      </c>
+      <c r="B24" s="8"/>
+      <c r="C24" s="8" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="7" t="s">
+        <v>262</v>
+      </c>
+      <c r="B25" s="6"/>
+      <c r="C25" s="6" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="B26" s="6"/>
+      <c r="C26" s="6" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="B27" s="6"/>
+      <c r="C27" s="6" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="9" t="s">
+        <v>265</v>
+      </c>
+      <c r="B28" s="8"/>
+      <c r="C28" s="8" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="B29" s="8"/>
+      <c r="C29" s="8" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="8" t="s">
+        <v>267</v>
+      </c>
+      <c r="B30" s="8"/>
+      <c r="C30" s="8" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="8" t="s">
+        <v>268</v>
+      </c>
+      <c r="B31" s="8"/>
+      <c r="C31" s="8" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="B32" s="8"/>
+      <c r="C32" s="8" t="s">
+        <v>274</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Some fix in manure excretion data + use animal_NIR rel.
</commit_message>
<xml_diff>
--- a/data/relation_tables.xlsx
+++ b/data/relation_tables.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="719" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="719" uniqueCount="276">
   <si>
     <t>CPC</t>
   </si>
@@ -841,13 +841,16 @@
     <t>horses</t>
   </si>
   <si>
-    <t>other pigs</t>
-  </si>
-  <si>
     <t>pigs for meat</t>
   </si>
   <si>
-    <t>other poultry</t>
+    <t>baors</t>
+  </si>
+  <si>
+    <t>chickens</t>
+  </si>
+  <si>
+    <t>laying hens</t>
   </si>
 </sst>
 </file>
@@ -2677,7 +2680,7 @@
       </c>
       <c r="B14" s="8"/>
       <c r="C14" s="8" t="s">
-        <v>270</v>
+        <v>251</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -2722,7 +2725,7 @@
       </c>
       <c r="B19" s="8"/>
       <c r="C19" s="8" t="s">
-        <v>272</v>
+        <v>256</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -2731,7 +2734,7 @@
       </c>
       <c r="B20" s="8"/>
       <c r="C20" s="8" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -2740,7 +2743,7 @@
       </c>
       <c r="B21" s="8"/>
       <c r="C21" s="8" t="s">
-        <v>272</v>
+        <v>258</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -2749,7 +2752,7 @@
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="8" t="s">
-        <v>272</v>
+        <v>256</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -2758,7 +2761,7 @@
       </c>
       <c r="B23" s="8"/>
       <c r="C23" s="8" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -2767,7 +2770,7 @@
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="8" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -2785,7 +2788,7 @@
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -2794,7 +2797,7 @@
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -2812,7 +2815,7 @@
       </c>
       <c r="B29" s="8"/>
       <c r="C29" s="8" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -2821,7 +2824,7 @@
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="8" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -2830,7 +2833,7 @@
       </c>
       <c r="B31" s="8"/>
       <c r="C31" s="8" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -2839,7 +2842,7 @@
       </c>
       <c r="B32" s="8"/>
       <c r="C32" s="8" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixxed spelling of 'boar'
</commit_message>
<xml_diff>
--- a/data/relation_tables.xlsx
+++ b/data/relation_tables.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="719" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="719" uniqueCount="275">
   <si>
     <t>CPC</t>
   </si>
@@ -842,9 +842,6 @@
   </si>
   <si>
     <t>pigs for meat</t>
-  </si>
-  <si>
-    <t>baors</t>
   </si>
   <si>
     <t>chickens</t>
@@ -2734,7 +2731,7 @@
       </c>
       <c r="B20" s="8"/>
       <c r="C20" s="8" t="s">
-        <v>273</v>
+        <v>257</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -2788,7 +2785,7 @@
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="6" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -2797,7 +2794,7 @@
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="6" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -2806,7 +2803,7 @@
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="8" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -2815,7 +2812,7 @@
       </c>
       <c r="B29" s="8"/>
       <c r="C29" s="8" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -2824,7 +2821,7 @@
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="8" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -2833,7 +2830,7 @@
       </c>
       <c r="B31" s="8"/>
       <c r="C31" s="8" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -2842,7 +2839,7 @@
       </c>
       <c r="B32" s="8"/>
       <c r="C32" s="8" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added missing feeds and by_prods to relation tables
</commit_message>
<xml_diff>
--- a/data/relation_tables.xlsx
+++ b/data/relation_tables.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="crop" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="719" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="278">
   <si>
     <t>CPC</t>
   </si>
@@ -848,6 +848,15 @@
   </si>
   <si>
     <t>laying hens</t>
+  </si>
+  <si>
+    <t>minerals</t>
+  </si>
+  <si>
+    <t>maize gluten meal</t>
+  </si>
+  <si>
+    <t>cream</t>
   </si>
 </sst>
 </file>
@@ -3720,7 +3729,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:B44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
@@ -3911,9 +3920,9 @@
         <v>187</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>167</v>
+    <row r="24" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>208</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>187</v>
@@ -3921,7 +3930,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>187</v>
@@ -3929,7 +3938,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>187</v>
@@ -3937,7 +3946,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>187</v>
@@ -3945,7 +3954,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>187</v>
@@ -3953,7 +3962,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>187</v>
@@ -3961,7 +3970,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>187</v>
@@ -3969,7 +3978,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>187</v>
@@ -3977,7 +3986,7 @@
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>187</v>
@@ -3985,31 +3994,31 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>176</v>
-      </c>
-      <c r="B33" t="s">
-        <v>188</v>
+        <v>175</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>177</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>187</v>
+        <v>176</v>
+      </c>
+      <c r="B34" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>179</v>
+        <v>187</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
+        <v>276</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>187</v>
@@ -4017,7 +4026,7 @@
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>188</v>
@@ -4025,7 +4034,7 @@
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>187</v>
@@ -4033,36 +4042,61 @@
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>187</v>
       </c>
     </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>183</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>184</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>275</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>187</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
@@ -4192,17 +4226,17 @@
         <v>210</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>224</v>
+        <v>276</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>183</v>
+        <v>224</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>212</v>
@@ -4210,7 +4244,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>212</v>
@@ -4218,7 +4252,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>208</v>
+        <v>182</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>212</v>
@@ -4226,7 +4260,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>166</v>
+        <v>208</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>212</v>
@@ -4234,31 +4268,31 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>217</v>
+        <v>166</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>216</v>
+        <v>164</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>178</v>
+        <v>165</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>179</v>
+        <v>168</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>212</v>
@@ -4266,65 +4300,121 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>167</v>
+        <v>217</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>229</v>
+        <v>216</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>230</v>
+        <v>178</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>226</v>
+        <v>179</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>225</v>
+        <v>167</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B34" s="1" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+    <row r="35" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>232</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B36" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
         <v>233</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B37" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>169</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>184</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>212</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updates default data to be compatible w. MFF scenarios
</commit_message>
<xml_diff>
--- a/data/relation_tables.xlsx
+++ b/data/relation_tables.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A094C2C-C155-4179-9196-90C5E8A32CC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="4"/>
+    <workbookView xWindow="3945" yWindow="1815" windowWidth="21600" windowHeight="11295" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="crop" sheetId="1" r:id="rId1"/>
@@ -13,17 +14,28 @@
     <sheet name="feed" sheetId="3" r:id="rId4"/>
     <sheet name="by_prod" sheetId="4" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="747" uniqueCount="282">
   <si>
     <t>CPC</t>
   </si>
@@ -857,12 +869,24 @@
   </si>
   <si>
     <t>cream</t>
+  </si>
+  <si>
+    <t>grass meal</t>
+  </si>
+  <si>
+    <t>pea protein</t>
+  </si>
+  <si>
+    <t>black soldier fly larvae meal</t>
+  </si>
+  <si>
+    <t>black soldier fly larvae</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -924,12 +948,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
@@ -1214,1314 +1236,1314 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F65"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="23" style="1" customWidth="1"/>
+    <col min="4" max="5" width="23" customWidth="1"/>
     <col min="6" max="6" width="22.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" t="s">
         <v>130</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" t="s">
         <v>130</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" t="s">
         <v>130</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" t="s">
         <v>130</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" t="s">
         <v>130</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" t="s">
         <v>130</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" t="s">
         <v>130</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" t="s">
         <v>130</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" t="s">
         <v>130</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" t="s">
         <v>130</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" t="s">
         <v>130</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" t="s">
         <v>130</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F7" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="A8" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" t="s">
         <v>6</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D8" t="s">
         <v>130</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" t="s">
         <v>130</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="F8" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="A9" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D9" t="s">
         <v>130</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E9" t="s">
         <v>130</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="F9" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="A10" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" t="s">
         <v>130</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" t="s">
         <v>130</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="F10" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+      <c r="A11" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" t="s">
         <v>10</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="D11" t="s">
         <v>130</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E11" t="s">
         <v>130</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="F11" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="A12" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" t="s">
         <v>29</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="D12" t="s">
         <v>133</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="E12" t="s">
         <v>191</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="F12" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+      <c r="A13" t="s">
         <v>31</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" t="s">
         <v>30</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="D13" t="s">
         <v>133</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="E13" t="s">
         <v>191</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="F13" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+      <c r="A14" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" t="s">
         <v>29</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="D14" t="s">
         <v>133</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="E14" t="s">
         <v>191</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="F14" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
+      <c r="A15" t="s">
         <v>35</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" t="s">
         <v>34</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" t="s">
         <v>29</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="D15" t="s">
         <v>133</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="E15" t="s">
         <v>191</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="F15" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+      <c r="A16" t="s">
         <v>37</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" t="s">
         <v>36</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" t="s">
         <v>38</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="D16" t="s">
         <v>133</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="E16" t="s">
         <v>191</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="F16" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
+      <c r="A17" t="s">
         <v>40</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" t="s">
         <v>39</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" t="s">
         <v>38</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="D17" t="s">
         <v>133</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="E17" t="s">
         <v>191</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="F17" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
+      <c r="A18" t="s">
         <v>42</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" t="s">
         <v>41</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" t="s">
         <v>43</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="D18" t="s">
         <v>133</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="E18" t="s">
         <v>191</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="F18" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
+      <c r="A19" t="s">
         <v>45</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" t="s">
         <v>44</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" t="s">
         <v>43</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="D19" t="s">
         <v>133</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="E19" t="s">
         <v>191</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="F19" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
+      <c r="A20" t="s">
         <v>47</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" t="s">
         <v>46</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" t="s">
         <v>47</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="D20" t="s">
         <v>133</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="E20" t="s">
         <v>191</v>
       </c>
-      <c r="F20" s="1" t="s">
+      <c r="F20" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
+      <c r="A21" t="s">
         <v>49</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C21" t="s">
         <v>50</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="D21" t="s">
         <v>68</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="E21" t="s">
         <v>191</v>
       </c>
-      <c r="F21" s="1" t="s">
+      <c r="F21" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
+      <c r="A22" t="s">
         <v>52</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" t="s">
         <v>51</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C22" t="s">
         <v>52</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="D22" t="s">
         <v>52</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="E22" t="s">
         <v>192</v>
       </c>
-      <c r="F22" s="1" t="s">
+      <c r="F22" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
+      <c r="A23" t="s">
         <v>54</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" t="s">
         <v>53</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C23" t="s">
         <v>55</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="D23" t="s">
         <v>133</v>
       </c>
-      <c r="E23" s="1" t="s">
+      <c r="E23" t="s">
         <v>191</v>
       </c>
-      <c r="F23" s="1" t="s">
+      <c r="F23" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
+      <c r="A24" t="s">
         <v>57</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" t="s">
         <v>56</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="C24" t="s">
         <v>55</v>
       </c>
-      <c r="D24" s="1" t="s">
+      <c r="D24" t="s">
         <v>133</v>
       </c>
-      <c r="E24" s="1" t="s">
+      <c r="E24" t="s">
         <v>191</v>
       </c>
-      <c r="F24" s="1" t="s">
+      <c r="F24" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
+      <c r="A25" t="s">
         <v>59</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B25" t="s">
         <v>58</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="C25" t="s">
         <v>59</v>
       </c>
-      <c r="D25" s="1" t="s">
+      <c r="D25" t="s">
         <v>68</v>
       </c>
-      <c r="E25" s="1" t="s">
+      <c r="E25" t="s">
         <v>191</v>
       </c>
-      <c r="F25" s="1" t="s">
+      <c r="F25" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
+      <c r="A26" t="s">
         <v>61</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" t="s">
         <v>60</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C26" t="s">
         <v>50</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D26" t="s">
         <v>68</v>
       </c>
-      <c r="E26" s="1" t="s">
+      <c r="E26" t="s">
         <v>61</v>
       </c>
-      <c r="F26" s="1" t="s">
+      <c r="F26" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
+      <c r="A27" t="s">
         <v>63</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" t="s">
         <v>62</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="C27" t="s">
         <v>50</v>
       </c>
-      <c r="D27" s="1" t="s">
+      <c r="D27" t="s">
         <v>68</v>
       </c>
-      <c r="E27" s="1" t="s">
+      <c r="E27" t="s">
         <v>63</v>
       </c>
-      <c r="F27" s="1" t="s">
+      <c r="F27" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
+      <c r="A28" t="s">
         <v>65</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" t="s">
         <v>64</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="C28" t="s">
         <v>50</v>
       </c>
-      <c r="D28" s="1" t="s">
+      <c r="D28" t="s">
         <v>68</v>
       </c>
-      <c r="E28" s="1" t="s">
+      <c r="E28" t="s">
         <v>192</v>
       </c>
-      <c r="F28" s="1" t="s">
+      <c r="F28" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
+      <c r="A29" t="s">
         <v>67</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B29" t="s">
         <v>66</v>
       </c>
-      <c r="C29" s="1" t="s">
+      <c r="C29" t="s">
         <v>68</v>
       </c>
-      <c r="D29" s="1" t="s">
+      <c r="D29" t="s">
         <v>68</v>
       </c>
-      <c r="E29" s="1" t="s">
+      <c r="E29" t="s">
         <v>191</v>
       </c>
-      <c r="F29" s="1" t="s">
+      <c r="F29" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
+      <c r="A30" t="s">
         <v>70</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B30" t="s">
         <v>69</v>
       </c>
-      <c r="C30" s="1" t="s">
+      <c r="C30" t="s">
         <v>68</v>
       </c>
-      <c r="D30" s="1" t="s">
+      <c r="D30" t="s">
         <v>68</v>
       </c>
-      <c r="E30" s="1" t="s">
+      <c r="E30" t="s">
         <v>191</v>
       </c>
-      <c r="F30" s="1" t="s">
+      <c r="F30" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
+      <c r="A31" t="s">
         <v>72</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B31" t="s">
         <v>71</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="C31" t="s">
         <v>68</v>
       </c>
-      <c r="D31" s="1" t="s">
+      <c r="D31" t="s">
         <v>68</v>
       </c>
-      <c r="E31" s="1" t="s">
+      <c r="E31" t="s">
         <v>191</v>
       </c>
-      <c r="F31" s="1" t="s">
+      <c r="F31" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
+      <c r="A32" t="s">
         <v>74</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B32" t="s">
         <v>73</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="C32" t="s">
         <v>74</v>
       </c>
-      <c r="D32" s="1" t="s">
+      <c r="D32" t="s">
         <v>75</v>
       </c>
-      <c r="E32" s="1" t="s">
+      <c r="E32" t="s">
         <v>192</v>
       </c>
-      <c r="F32" s="1" t="s">
+      <c r="F32" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="33" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="1" t="s">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
         <v>193</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B33" t="s">
         <v>73</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="C33" t="s">
         <v>74</v>
       </c>
-      <c r="D33" s="1" t="s">
+      <c r="D33" t="s">
         <v>75</v>
       </c>
-      <c r="E33" s="1" t="s">
+      <c r="E33" t="s">
         <v>192</v>
       </c>
-      <c r="F33" s="1" t="s">
+      <c r="F33" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="34" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="1" t="s">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>194</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B34" t="s">
         <v>73</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="C34" t="s">
         <v>74</v>
       </c>
-      <c r="D34" s="1" t="s">
+      <c r="D34" t="s">
         <v>75</v>
       </c>
-      <c r="E34" s="1" t="s">
+      <c r="E34" t="s">
         <v>192</v>
       </c>
-      <c r="F34" s="1" t="s">
+      <c r="F34" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" s="1" t="s">
+      <c r="A35" t="s">
         <v>78</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B35" t="s">
         <v>77</v>
       </c>
-      <c r="C35" s="1" t="s">
+      <c r="C35" t="s">
         <v>78</v>
       </c>
-      <c r="D35" s="1" t="s">
+      <c r="D35" t="s">
         <v>75</v>
       </c>
-      <c r="E35" s="1" t="s">
+      <c r="E35" t="s">
         <v>192</v>
       </c>
-      <c r="F35" s="1" t="s">
+      <c r="F35" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A36" s="1" t="s">
+      <c r="A36" t="s">
         <v>80</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B36" t="s">
         <v>79</v>
       </c>
-      <c r="C36" s="1" t="s">
+      <c r="C36" t="s">
         <v>81</v>
       </c>
-      <c r="D36" s="1" t="s">
+      <c r="D36" t="s">
         <v>131</v>
       </c>
-      <c r="E36" s="1" t="s">
+      <c r="E36" t="s">
         <v>191</v>
       </c>
-      <c r="F36" s="1" t="s">
+      <c r="F36" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" s="1" t="s">
+      <c r="A37" t="s">
         <v>83</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="B37" t="s">
         <v>82</v>
       </c>
-      <c r="C37" s="1" t="s">
+      <c r="C37" t="s">
         <v>81</v>
       </c>
-      <c r="D37" s="1" t="s">
+      <c r="D37" t="s">
         <v>131</v>
       </c>
-      <c r="E37" s="1" t="s">
+      <c r="E37" t="s">
         <v>191</v>
       </c>
-      <c r="F37" s="1" t="s">
+      <c r="F37" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A38" s="1" t="s">
+      <c r="A38" t="s">
         <v>85</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="B38" t="s">
         <v>84</v>
       </c>
-      <c r="C38" s="1" t="s">
+      <c r="C38" t="s">
         <v>81</v>
       </c>
-      <c r="D38" s="1" t="s">
+      <c r="D38" t="s">
         <v>131</v>
       </c>
-      <c r="E38" s="1" t="s">
+      <c r="E38" t="s">
         <v>191</v>
       </c>
-      <c r="F38" s="1" t="s">
+      <c r="F38" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" s="1" t="s">
+      <c r="A39" t="s">
         <v>87</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="B39" t="s">
         <v>86</v>
       </c>
-      <c r="C39" s="1" t="s">
+      <c r="C39" t="s">
         <v>81</v>
       </c>
-      <c r="D39" s="1" t="s">
+      <c r="D39" t="s">
         <v>131</v>
       </c>
-      <c r="E39" s="1" t="s">
+      <c r="E39" t="s">
         <v>191</v>
       </c>
-      <c r="F39" s="1" t="s">
+      <c r="F39" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="1" t="s">
+      <c r="A40" t="s">
         <v>89</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="B40" t="s">
         <v>88</v>
       </c>
-      <c r="C40" s="1" t="s">
+      <c r="C40" t="s">
         <v>81</v>
       </c>
-      <c r="D40" s="1" t="s">
+      <c r="D40" t="s">
         <v>131</v>
       </c>
-      <c r="E40" s="1" t="s">
+      <c r="E40" t="s">
         <v>191</v>
       </c>
-      <c r="F40" s="1" t="s">
+      <c r="F40" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" s="1" t="s">
+      <c r="A41" t="s">
         <v>91</v>
       </c>
-      <c r="B41" s="1" t="s">
+      <c r="B41" t="s">
         <v>90</v>
       </c>
-      <c r="C41" s="1" t="s">
+      <c r="C41" t="s">
         <v>81</v>
       </c>
-      <c r="D41" s="1" t="s">
+      <c r="D41" t="s">
         <v>131</v>
       </c>
-      <c r="E41" s="1" t="s">
+      <c r="E41" t="s">
         <v>191</v>
       </c>
-      <c r="F41" s="1" t="s">
+      <c r="F41" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42" s="1" t="s">
+      <c r="A42" t="s">
         <v>93</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="B42" t="s">
         <v>92</v>
       </c>
-      <c r="C42" s="1" t="s">
+      <c r="C42" t="s">
         <v>81</v>
       </c>
-      <c r="D42" s="1" t="s">
+      <c r="D42" t="s">
         <v>131</v>
       </c>
-      <c r="E42" s="1" t="s">
+      <c r="E42" t="s">
         <v>191</v>
       </c>
-      <c r="F42" s="1" t="s">
+      <c r="F42" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43" s="1" t="s">
+      <c r="A43" t="s">
         <v>95</v>
       </c>
-      <c r="B43" s="1" t="s">
+      <c r="B43" t="s">
         <v>94</v>
       </c>
-      <c r="C43" s="1" t="s">
+      <c r="C43" t="s">
         <v>81</v>
       </c>
-      <c r="D43" s="1" t="s">
+      <c r="D43" t="s">
         <v>131</v>
       </c>
-      <c r="E43" s="1" t="s">
+      <c r="E43" t="s">
         <v>191</v>
       </c>
-      <c r="F43" s="1" t="s">
+      <c r="F43" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" s="1" t="s">
+      <c r="A44" t="s">
         <v>97</v>
       </c>
-      <c r="B44" s="1" t="s">
+      <c r="B44" t="s">
         <v>96</v>
       </c>
-      <c r="C44" s="1" t="s">
+      <c r="C44" t="s">
         <v>81</v>
       </c>
-      <c r="D44" s="1" t="s">
+      <c r="D44" t="s">
         <v>131</v>
       </c>
-      <c r="E44" s="1" t="s">
+      <c r="E44" t="s">
         <v>191</v>
       </c>
-      <c r="F44" s="1" t="s">
+      <c r="F44" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="1" t="s">
+      <c r="A45" t="s">
         <v>99</v>
       </c>
-      <c r="B45" s="1" t="s">
+      <c r="B45" t="s">
         <v>98</v>
       </c>
-      <c r="C45" s="1" t="s">
+      <c r="C45" t="s">
         <v>100</v>
       </c>
-      <c r="D45" s="1" t="s">
+      <c r="D45" t="s">
         <v>131</v>
       </c>
-      <c r="E45" s="1" t="s">
+      <c r="E45" t="s">
         <v>191</v>
       </c>
-      <c r="F45" s="1" t="s">
+      <c r="F45" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A46" s="1" t="s">
+      <c r="A46" t="s">
         <v>102</v>
       </c>
-      <c r="B46" s="1" t="s">
+      <c r="B46" t="s">
         <v>101</v>
       </c>
-      <c r="C46" s="1" t="s">
+      <c r="C46" t="s">
         <v>100</v>
       </c>
-      <c r="D46" s="1" t="s">
+      <c r="D46" t="s">
         <v>131</v>
       </c>
-      <c r="E46" s="1" t="s">
+      <c r="E46" t="s">
         <v>191</v>
       </c>
-      <c r="F46" s="1" t="s">
+      <c r="F46" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47" s="1" t="s">
+      <c r="A47" t="s">
         <v>104</v>
       </c>
-      <c r="B47" s="1" t="s">
+      <c r="B47" t="s">
         <v>103</v>
       </c>
-      <c r="C47" s="1" t="s">
+      <c r="C47" t="s">
         <v>100</v>
       </c>
-      <c r="D47" s="1" t="s">
+      <c r="D47" t="s">
         <v>131</v>
       </c>
-      <c r="E47" s="1" t="s">
+      <c r="E47" t="s">
         <v>191</v>
       </c>
-      <c r="F47" s="1" t="s">
+      <c r="F47" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A48" s="1" t="s">
+      <c r="A48" t="s">
         <v>106</v>
       </c>
-      <c r="B48" s="1" t="s">
+      <c r="B48" t="s">
         <v>105</v>
       </c>
-      <c r="C48" s="1" t="s">
+      <c r="C48" t="s">
         <v>107</v>
       </c>
-      <c r="D48" s="1" t="s">
+      <c r="D48" t="s">
         <v>131</v>
       </c>
-      <c r="E48" s="1" t="s">
+      <c r="E48" t="s">
         <v>191</v>
       </c>
-      <c r="F48" s="1" t="s">
+      <c r="F48" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A49" s="1" t="s">
+      <c r="A49" t="s">
         <v>109</v>
       </c>
-      <c r="B49" s="1" t="s">
+      <c r="B49" t="s">
         <v>108</v>
       </c>
-      <c r="C49" s="1" t="s">
+      <c r="C49" t="s">
         <v>107</v>
       </c>
-      <c r="D49" s="1" t="s">
+      <c r="D49" t="s">
         <v>131</v>
       </c>
-      <c r="E49" s="1" t="s">
+      <c r="E49" t="s">
         <v>191</v>
       </c>
-      <c r="F49" s="1" t="s">
+      <c r="F49" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A50" s="1" t="s">
+      <c r="A50" t="s">
         <v>111</v>
       </c>
-      <c r="B50" s="1" t="s">
+      <c r="B50" t="s">
         <v>110</v>
       </c>
-      <c r="C50" s="1" t="s">
+      <c r="C50" t="s">
         <v>107</v>
       </c>
-      <c r="D50" s="1" t="s">
+      <c r="D50" t="s">
         <v>131</v>
       </c>
-      <c r="E50" s="1" t="s">
+      <c r="E50" t="s">
         <v>191</v>
       </c>
-      <c r="F50" s="1" t="s">
+      <c r="F50" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" s="1" t="s">
+      <c r="A51" t="s">
         <v>113</v>
       </c>
-      <c r="B51" s="1" t="s">
+      <c r="B51" t="s">
         <v>112</v>
       </c>
-      <c r="C51" s="1" t="s">
+      <c r="C51" t="s">
         <v>114</v>
       </c>
-      <c r="D51" s="1" t="s">
+      <c r="D51" t="s">
         <v>132</v>
       </c>
-      <c r="E51" s="1" t="s">
+      <c r="E51" t="s">
         <v>192</v>
       </c>
-      <c r="F51" s="1" t="s">
+      <c r="F51" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A52" s="1" t="s">
+      <c r="A52" t="s">
         <v>117</v>
       </c>
-      <c r="B52" s="1" t="s">
+      <c r="B52" t="s">
         <v>116</v>
       </c>
-      <c r="C52" s="1" t="s">
+      <c r="C52" t="s">
         <v>114</v>
       </c>
-      <c r="D52" s="1" t="s">
+      <c r="D52" t="s">
         <v>132</v>
       </c>
-      <c r="E52" s="1" t="s">
+      <c r="E52" t="s">
         <v>192</v>
       </c>
-      <c r="F52" s="1" t="s">
+      <c r="F52" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A53" s="1" t="s">
+      <c r="A53" t="s">
         <v>119</v>
       </c>
-      <c r="B53" s="1" t="s">
+      <c r="B53" t="s">
         <v>118</v>
       </c>
-      <c r="C53" s="1" t="s">
+      <c r="C53" t="s">
         <v>114</v>
       </c>
-      <c r="D53" s="1" t="s">
+      <c r="D53" t="s">
         <v>132</v>
       </c>
-      <c r="E53" s="1" t="s">
+      <c r="E53" t="s">
         <v>192</v>
       </c>
-      <c r="F53" s="1" t="s">
+      <c r="F53" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A54" s="1" t="s">
+      <c r="A54" t="s">
         <v>121</v>
       </c>
-      <c r="B54" s="1" t="s">
+      <c r="B54" t="s">
         <v>120</v>
       </c>
-      <c r="C54" s="1" t="s">
+      <c r="C54" t="s">
         <v>114</v>
       </c>
-      <c r="D54" s="1" t="s">
+      <c r="D54" t="s">
         <v>132</v>
       </c>
-      <c r="E54" s="1" t="s">
+      <c r="E54" t="s">
         <v>192</v>
       </c>
-      <c r="F54" s="1" t="s">
+      <c r="F54" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A55" s="1" t="s">
+      <c r="A55" t="s">
         <v>123</v>
       </c>
-      <c r="B55" s="1" t="s">
+      <c r="B55" t="s">
         <v>122</v>
       </c>
-      <c r="C55" s="1" t="s">
+      <c r="C55" t="s">
         <v>114</v>
       </c>
-      <c r="D55" s="1" t="s">
+      <c r="D55" t="s">
         <v>132</v>
       </c>
-      <c r="E55" s="1" t="s">
+      <c r="E55" t="s">
         <v>192</v>
       </c>
-      <c r="F55" s="1" t="s">
+      <c r="F55" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A56" s="1" t="s">
+      <c r="A56" t="s">
         <v>125</v>
       </c>
-      <c r="B56" s="1" t="s">
+      <c r="B56" t="s">
         <v>124</v>
       </c>
-      <c r="C56" s="1" t="s">
+      <c r="C56" t="s">
         <v>126</v>
       </c>
-      <c r="D56" s="1" t="s">
+      <c r="D56" t="s">
         <v>132</v>
       </c>
-      <c r="E56" s="1" t="s">
+      <c r="E56" t="s">
         <v>192</v>
       </c>
-      <c r="F56" s="1" t="s">
+      <c r="F56" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A57" s="1" t="s">
+      <c r="A57" t="s">
         <v>128</v>
       </c>
-      <c r="B57" s="1" t="s">
+      <c r="B57" t="s">
         <v>127</v>
       </c>
-      <c r="C57" s="1" t="s">
+      <c r="C57" t="s">
         <v>126</v>
       </c>
-      <c r="D57" s="1" t="s">
+      <c r="D57" t="s">
         <v>132</v>
       </c>
-      <c r="E57" s="1" t="s">
+      <c r="E57" t="s">
         <v>192</v>
       </c>
-      <c r="F57" s="1" t="s">
+      <c r="F57" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A58" s="3" t="s">
+      <c r="A58" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="B58" s="3" t="s">
+      <c r="B58" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="C58" s="3" t="s">
+      <c r="C58" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D58" s="3" t="s">
+      <c r="D58" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="E58" s="3" t="s">
+      <c r="E58" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="F58" s="3" t="s">
+      <c r="F58" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A59" s="3" t="s">
+      <c r="A59" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="B59" s="3" t="s">
+      <c r="B59" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="C59" s="3" t="s">
+      <c r="C59" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D59" s="3" t="s">
+      <c r="D59" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="E59" s="3" t="s">
+      <c r="E59" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="F59" s="3" t="s">
+      <c r="F59" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A60" s="4" t="s">
+      <c r="A60" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="B60" s="4" t="s">
+      <c r="B60" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="C60" s="4" t="s">
+      <c r="C60" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D60" s="4" t="s">
+      <c r="D60" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="E60" s="4" t="s">
+      <c r="E60" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="F60" s="4" t="s">
+      <c r="F60" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A61" s="3" t="s">
+      <c r="A61" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="B61" s="3" t="s">
+      <c r="B61" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="C61" s="3" t="s">
+      <c r="C61" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D61" s="3" t="s">
+      <c r="D61" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="E61" s="3" t="s">
+      <c r="E61" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="F61" s="3" t="s">
+      <c r="F61" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A62" s="3" t="s">
+      <c r="A62" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="B62" s="3" t="s">
+      <c r="B62" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="C62" s="3" t="s">
+      <c r="C62" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D62" s="3" t="s">
+      <c r="D62" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="E62" s="3" t="s">
+      <c r="E62" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="F62" s="3" t="s">
+      <c r="F62" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A63" s="3" t="s">
+      <c r="A63" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="B63" s="3" t="s">
+      <c r="B63" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="C63" s="3" t="s">
+      <c r="C63" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="D63" s="3" t="s">
+      <c r="D63" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="E63" s="3" t="s">
+      <c r="E63" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="F63" s="3" t="s">
+      <c r="F63" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A64" s="3" t="s">
+      <c r="A64" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="B64" s="3" t="s">
+      <c r="B64" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="C64" s="3" t="s">
+      <c r="C64" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="D64" s="3" t="s">
+      <c r="D64" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="E64" s="3" t="s">
+      <c r="E64" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="F64" s="3" t="s">
+      <c r="F64" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A65" s="3" t="s">
+      <c r="A65" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="B65" s="3" t="s">
+      <c r="B65" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="C65" s="3" t="s">
+      <c r="C65" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="D65" s="3" t="s">
+      <c r="D65" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="E65" s="3" t="s">
+      <c r="E65" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="F65" s="3" t="s">
+      <c r="F65" s="2" t="s">
         <v>7</v>
       </c>
     </row>
@@ -2532,7 +2554,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2542,312 +2564,312 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="3" t="s">
         <v>234</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="3" t="s">
         <v>246</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="3" t="s">
         <v>247</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="4" t="s">
         <v>236</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="4" t="s">
         <v>236</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="4" t="s">
         <v>236</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="4" t="s">
         <v>237</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="4" t="s">
         <v>237</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="4" t="s">
         <v>248</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="5" t="s">
         <v>241</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="5" t="s">
         <v>241</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="4" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="5" t="s">
         <v>242</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="4" t="s">
         <v>240</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="4" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="4" t="s">
         <v>243</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="5" t="s">
         <v>238</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="4" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="4" t="s">
         <v>244</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="4" t="s">
         <v>239</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="4" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="4" t="s">
         <v>245</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="4" t="s">
         <v>240</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="4" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="5" t="s">
         <v>238</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="5" t="s">
         <v>238</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="5" t="s">
         <v>238</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="4" t="s">
         <v>239</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="4" t="s">
         <v>239</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="4" t="s">
         <v>248</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="4" t="s">
         <v>240</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="4" t="s">
         <v>240</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="4" t="s">
         <v>248</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="6" t="s">
         <v>249</v>
       </c>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8" t="s">
+      <c r="B12" s="6"/>
+      <c r="C12" s="6" t="s">
         <v>270</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="6" t="s">
         <v>250</v>
       </c>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8" t="s">
+      <c r="B13" s="6"/>
+      <c r="C13" s="6" t="s">
         <v>270</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="6" t="s">
         <v>251</v>
       </c>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8" t="s">
+      <c r="B14" s="6"/>
+      <c r="C14" s="6" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="5" t="s">
         <v>252</v>
       </c>
-      <c r="B15" s="6"/>
-      <c r="C15" s="6" t="s">
+      <c r="B15" s="4"/>
+      <c r="C15" s="4" t="s">
         <v>271</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="s">
+      <c r="A16" s="4" t="s">
         <v>253</v>
       </c>
-      <c r="B16" s="6"/>
-      <c r="C16" s="6" t="s">
+      <c r="B16" s="4"/>
+      <c r="C16" s="4" t="s">
         <v>271</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="4" t="s">
         <v>254</v>
       </c>
-      <c r="B17" s="6"/>
-      <c r="C17" s="6" t="s">
+      <c r="B17" s="4"/>
+      <c r="C17" s="4" t="s">
         <v>271</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="4" t="s">
         <v>255</v>
       </c>
-      <c r="B18" s="6"/>
-      <c r="C18" s="6" t="s">
+      <c r="B18" s="4"/>
+      <c r="C18" s="4" t="s">
         <v>271</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="9" t="s">
+      <c r="A19" s="7" t="s">
         <v>256</v>
       </c>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8" t="s">
+      <c r="B19" s="6"/>
+      <c r="C19" s="6" t="s">
         <v>256</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="8" t="s">
+      <c r="A20" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="B20" s="8"/>
-      <c r="C20" s="8" t="s">
+      <c r="B20" s="6"/>
+      <c r="C20" s="6" t="s">
         <v>257</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="8" t="s">
+      <c r="A21" s="6" t="s">
         <v>258</v>
       </c>
-      <c r="B21" s="8"/>
-      <c r="C21" s="8" t="s">
+      <c r="B21" s="6"/>
+      <c r="C21" s="6" t="s">
         <v>258</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="8" t="s">
+      <c r="A22" s="6" t="s">
         <v>259</v>
       </c>
-      <c r="B22" s="8"/>
-      <c r="C22" s="8" t="s">
+      <c r="B22" s="6"/>
+      <c r="C22" s="6" t="s">
         <v>256</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="8" t="s">
+      <c r="A23" s="6" t="s">
         <v>260</v>
       </c>
-      <c r="B23" s="8"/>
-      <c r="C23" s="8" t="s">
+      <c r="B23" s="6"/>
+      <c r="C23" s="6" t="s">
         <v>272</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="8" t="s">
+      <c r="A24" s="6" t="s">
         <v>261</v>
       </c>
-      <c r="B24" s="8"/>
-      <c r="C24" s="8" t="s">
+      <c r="B24" s="6"/>
+      <c r="C24" s="6" t="s">
         <v>272</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="7" t="s">
+      <c r="A25" s="5" t="s">
         <v>262</v>
       </c>
-      <c r="B25" s="6"/>
-      <c r="C25" s="6" t="s">
+      <c r="B25" s="4"/>
+      <c r="C25" s="4" t="s">
         <v>262</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="6" t="s">
+      <c r="A26" s="4" t="s">
         <v>263</v>
       </c>
-      <c r="B26" s="6"/>
-      <c r="C26" s="6" t="s">
+      <c r="B26" s="4"/>
+      <c r="C26" s="4" t="s">
         <v>274</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="6" t="s">
+      <c r="A27" s="4" t="s">
         <v>264</v>
       </c>
-      <c r="B27" s="6"/>
-      <c r="C27" s="6" t="s">
+      <c r="B27" s="4"/>
+      <c r="C27" s="4" t="s">
         <v>274</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="9" t="s">
+      <c r="A28" s="7" t="s">
         <v>265</v>
       </c>
-      <c r="B28" s="8"/>
-      <c r="C28" s="8" t="s">
+      <c r="B28" s="6"/>
+      <c r="C28" s="6" t="s">
         <v>273</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="8" t="s">
+      <c r="A29" s="6" t="s">
         <v>266</v>
       </c>
-      <c r="B29" s="8"/>
-      <c r="C29" s="8" t="s">
+      <c r="B29" s="6"/>
+      <c r="C29" s="6" t="s">
         <v>274</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="8" t="s">
+      <c r="A30" s="6" t="s">
         <v>267</v>
       </c>
-      <c r="B30" s="8"/>
-      <c r="C30" s="8" t="s">
+      <c r="B30" s="6"/>
+      <c r="C30" s="6" t="s">
         <v>274</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="8" t="s">
+      <c r="A31" s="6" t="s">
         <v>268</v>
       </c>
-      <c r="B31" s="8"/>
-      <c r="C31" s="8" t="s">
+      <c r="B31" s="6"/>
+      <c r="C31" s="6" t="s">
         <v>274</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="8" t="s">
+      <c r="A32" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="B32" s="8"/>
-      <c r="C32" s="8" t="s">
+      <c r="B32" s="6"/>
+      <c r="C32" s="6" t="s">
         <v>274</v>
       </c>
     </row>
@@ -2858,7 +2880,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B107"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2867,858 +2889,858 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
+      <c r="A2">
         <v>111</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
+      <c r="A3">
         <v>112</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="1">
+      <c r="A4">
         <v>311</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
+      <c r="A5">
         <v>312</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="1">
+      <c r="A6">
         <v>321</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
+      <c r="A7">
         <v>322</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="1">
+      <c r="A8">
         <v>411</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="1">
+      <c r="A9">
         <v>421</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="1">
+      <c r="A10">
         <v>422</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="1">
+      <c r="A11">
         <v>431</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="1">
+      <c r="A12">
         <v>511</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="1">
+      <c r="A13">
         <v>512</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="1">
+      <c r="A14">
         <v>513</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="1">
+      <c r="A15">
         <v>514</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="1">
+      <c r="A16">
         <v>515</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="1">
+      <c r="A17">
         <v>521</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="1">
+      <c r="A18">
         <v>611</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="1">
+      <c r="A19">
         <v>612</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="1">
+      <c r="A20">
         <v>621</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="1">
+      <c r="A21">
         <v>622</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="1">
+      <c r="A22">
         <v>711</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="1">
+      <c r="A23">
         <v>731</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="1">
+      <c r="A24">
         <v>811</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="1">
+      <c r="A25">
         <v>812</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B25" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="1">
+      <c r="A26">
         <v>813</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" s="1">
+      <c r="A27">
         <v>814</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="1">
+      <c r="A28">
         <v>821</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="1">
+      <c r="A29">
         <v>831</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B29" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" s="1">
+      <c r="A30">
         <v>911</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B30" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" s="1">
+      <c r="A31">
         <v>912</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B31" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" s="1">
+      <c r="A32">
         <v>913</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B32" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" s="1">
+      <c r="A33">
         <v>1011</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B33" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" s="1">
+      <c r="A34">
         <v>1111</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B34" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" s="1">
+      <c r="A35">
         <v>1112</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B35" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" s="1">
+      <c r="A36">
         <v>1121</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B36" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" s="1">
+      <c r="A37">
         <v>1122</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="B37" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" s="1">
+      <c r="A38">
         <v>1123</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="B38" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" s="1">
+      <c r="A39">
         <v>1124</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="B39" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40" s="1">
+      <c r="A40">
         <v>1131</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="B40" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41" s="1">
+      <c r="A41">
         <v>1211</v>
       </c>
-      <c r="B41" s="1" t="s">
+      <c r="B41" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" s="1">
+      <c r="A42">
         <v>1212</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="B42" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" s="1">
+      <c r="A43">
         <v>1213</v>
       </c>
-      <c r="B43" s="1" t="s">
+      <c r="B43" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A44" s="1">
+      <c r="A44">
         <v>1214</v>
       </c>
-      <c r="B44" s="1" t="s">
+      <c r="B44" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45" s="1">
+      <c r="A45">
         <v>1215</v>
       </c>
-      <c r="B45" s="1" t="s">
+      <c r="B45" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46" s="1">
+      <c r="A46">
         <v>1216</v>
       </c>
-      <c r="B46" s="1" t="s">
+      <c r="B46" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47" s="1">
+      <c r="A47">
         <v>1221</v>
       </c>
-      <c r="B47" s="1" t="s">
+      <c r="B47" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A48" s="1">
+      <c r="A48">
         <v>1222</v>
       </c>
-      <c r="B48" s="1" t="s">
+      <c r="B48" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A49" s="1">
+      <c r="A49">
         <v>1311</v>
       </c>
-      <c r="B49" s="1" t="s">
+      <c r="B49" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A50" s="1">
+      <c r="A50">
         <v>1321</v>
       </c>
-      <c r="B50" s="1" t="s">
+      <c r="B50" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A51" s="1">
+      <c r="A51">
         <v>1322</v>
       </c>
-      <c r="B51" s="1" t="s">
+      <c r="B51" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A52" s="1">
+      <c r="A52">
         <v>1331</v>
       </c>
-      <c r="B52" s="1" t="s">
+      <c r="B52" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A53" s="1">
+      <c r="A53">
         <v>1411</v>
       </c>
-      <c r="B53" s="1" t="s">
+      <c r="B53" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A54" s="1">
+      <c r="A54">
         <v>1412</v>
       </c>
-      <c r="B54" s="1" t="s">
+      <c r="B54" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A55" s="1">
+      <c r="A55">
         <v>1421</v>
       </c>
-      <c r="B55" s="1" t="s">
+      <c r="B55" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A56" s="1">
+      <c r="A56">
         <v>1511</v>
       </c>
-      <c r="B56" s="1" t="s">
+      <c r="B56" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A57" s="1">
+      <c r="A57">
         <v>1512</v>
       </c>
-      <c r="B57" s="1" t="s">
+      <c r="B57" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A58" s="1">
+      <c r="A58">
         <v>1521</v>
       </c>
-      <c r="B58" s="1" t="s">
+      <c r="B58" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A59" s="1">
+      <c r="A59">
         <v>1522</v>
       </c>
-      <c r="B59" s="1" t="s">
+      <c r="B59" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A60" s="1">
+      <c r="A60">
         <v>1611</v>
       </c>
-      <c r="B60" s="1" t="s">
+      <c r="B60" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A61" s="1">
+      <c r="A61">
         <v>1612</v>
       </c>
-      <c r="B61" s="1" t="s">
+      <c r="B61" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A62" s="1">
+      <c r="A62">
         <v>1613</v>
       </c>
-      <c r="B62" s="1" t="s">
+      <c r="B62" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A63" s="1">
+      <c r="A63">
         <v>1614</v>
       </c>
-      <c r="B63" s="1" t="s">
+      <c r="B63" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A64" s="1">
+      <c r="A64">
         <v>1615</v>
       </c>
-      <c r="B64" s="1" t="s">
+      <c r="B64" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A65" s="1">
+      <c r="A65">
         <v>1616</v>
       </c>
-      <c r="B65" s="1" t="s">
+      <c r="B65" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A66" s="1">
+      <c r="A66">
         <v>1617</v>
       </c>
-      <c r="B66" s="1" t="s">
+      <c r="B66" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A67" s="1">
+      <c r="A67">
         <v>1621</v>
       </c>
-      <c r="B67" s="1" t="s">
+      <c r="B67" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A68" s="1">
+      <c r="A68">
         <v>1622</v>
       </c>
-      <c r="B68" s="1" t="s">
+      <c r="B68" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A69" s="1">
+      <c r="A69">
         <v>1623</v>
       </c>
-      <c r="B69" s="1" t="s">
+      <c r="B69" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A70" s="1">
+      <c r="A70">
         <v>1711</v>
       </c>
-      <c r="B70" s="1" t="s">
+      <c r="B70" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A71" s="1">
+      <c r="A71">
         <v>1712</v>
       </c>
-      <c r="B71" s="1" t="s">
+      <c r="B71" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A72" s="1">
+      <c r="A72">
         <v>1713</v>
       </c>
-      <c r="B72" s="1" t="s">
+      <c r="B72" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A73" s="1">
+      <c r="A73">
         <v>1721</v>
       </c>
-      <c r="B73" s="1" t="s">
+      <c r="B73" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A74" s="1">
+      <c r="A74">
         <v>1722</v>
       </c>
-      <c r="B74" s="1" t="s">
+      <c r="B74" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A75" s="1">
+      <c r="A75">
         <v>1723</v>
       </c>
-      <c r="B75" s="1" t="s">
+      <c r="B75" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A76" s="1">
+      <c r="A76">
         <v>1724</v>
       </c>
-      <c r="B76" s="1" t="s">
+      <c r="B76" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A77" s="1">
+      <c r="A77">
         <v>1811</v>
       </c>
-      <c r="B77" s="1" t="s">
+      <c r="B77" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A78" s="1">
+      <c r="A78">
         <v>1812</v>
       </c>
-      <c r="B78" s="1" t="s">
+      <c r="B78" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A79" s="1">
+      <c r="A79">
         <v>1813</v>
       </c>
-      <c r="B79" s="1" t="s">
+      <c r="B79" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A80" s="1">
+      <c r="A80">
         <v>1821</v>
       </c>
-      <c r="B80" s="1" t="s">
+      <c r="B80" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A81" s="1">
+      <c r="A81">
         <v>1911</v>
       </c>
-      <c r="B81" s="1" t="s">
+      <c r="B81" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A82" s="1">
+      <c r="A82">
         <v>1912</v>
       </c>
-      <c r="B82" s="1" t="s">
+      <c r="B82" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A83" s="1">
+      <c r="A83">
         <v>1921</v>
       </c>
-      <c r="B83" s="1" t="s">
+      <c r="B83" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A84" s="1">
+      <c r="A84">
         <v>1922</v>
       </c>
-      <c r="B84" s="1" t="s">
+      <c r="B84" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A85" s="1">
+      <c r="A85">
         <v>2011</v>
       </c>
-      <c r="B85" s="1" t="s">
+      <c r="B85" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A86" s="1">
+      <c r="A86">
         <v>2012</v>
       </c>
-      <c r="B86" s="1" t="s">
+      <c r="B86" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A87" s="1">
+      <c r="A87">
         <v>2019</v>
       </c>
-      <c r="B87" s="1" t="s">
+      <c r="B87" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A88" s="1">
+      <c r="A88">
         <v>2111</v>
       </c>
-      <c r="B88" s="1" t="s">
+      <c r="B88" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A89" s="1">
+      <c r="A89">
         <v>2121</v>
       </c>
-      <c r="B89" s="1" t="s">
+      <c r="B89" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A90" s="1">
+      <c r="A90">
         <v>2122</v>
       </c>
-      <c r="B90" s="1" t="s">
+      <c r="B90" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A91" s="1">
+      <c r="A91">
         <v>2211</v>
       </c>
-      <c r="B91" s="1" t="s">
+      <c r="B91" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A92" s="1">
+      <c r="A92">
         <v>2212</v>
       </c>
-      <c r="B92" s="1" t="s">
+      <c r="B92" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A93" s="1">
+      <c r="A93">
         <v>2221</v>
       </c>
-      <c r="B93" s="1" t="s">
+      <c r="B93" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A94" s="1">
+      <c r="A94">
         <v>2311</v>
       </c>
-      <c r="B94" s="1" t="s">
+      <c r="B94" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A95" s="1">
+      <c r="A95">
         <v>2312</v>
       </c>
-      <c r="B95" s="1" t="s">
+      <c r="B95" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A96" s="1">
+      <c r="A96">
         <v>2319</v>
       </c>
-      <c r="B96" s="1" t="s">
+      <c r="B96" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A97" s="1">
+      <c r="A97">
         <v>2331</v>
       </c>
-      <c r="B97" s="1" t="s">
+      <c r="B97" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A98" s="1">
+      <c r="A98">
         <v>2411</v>
       </c>
-      <c r="B98" s="1" t="s">
+      <c r="B98" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A99" s="1">
+      <c r="A99">
         <v>2412</v>
       </c>
-      <c r="B99" s="1" t="s">
+      <c r="B99" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A100" s="1">
+      <c r="A100">
         <v>2413</v>
       </c>
-      <c r="B100" s="1" t="s">
+      <c r="B100" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A101" s="1">
+      <c r="A101">
         <v>2414</v>
       </c>
-      <c r="B101" s="1" t="s">
+      <c r="B101" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A102" s="1">
+      <c r="A102">
         <v>2415</v>
       </c>
-      <c r="B102" s="1" t="s">
+      <c r="B102" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A103" s="1">
+      <c r="A103">
         <v>2419</v>
       </c>
-      <c r="B103" s="1" t="s">
+      <c r="B103" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A104" s="1">
+      <c r="A104">
         <v>2511</v>
       </c>
-      <c r="B104" s="1" t="s">
+      <c r="B104" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A105" s="1">
+      <c r="A105">
         <v>2512</v>
       </c>
-      <c r="B105" s="1" t="s">
+      <c r="B105" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A106" s="1">
+      <c r="A106">
         <v>2519</v>
       </c>
-      <c r="B106" s="1" t="s">
+      <c r="B106" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A107" s="1">
+      <c r="A107">
         <v>2521</v>
       </c>
-      <c r="B107" s="1" t="s">
+      <c r="B107" t="s">
         <v>143</v>
       </c>
     </row>
@@ -3728,8 +3750,8 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B44"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:B47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
@@ -3737,10 +3759,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>185</v>
       </c>
     </row>
@@ -3756,7 +3778,7 @@
       <c r="A3" t="s">
         <v>146</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>186</v>
       </c>
     </row>
@@ -3764,7 +3786,7 @@
       <c r="A4" t="s">
         <v>147</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>147</v>
       </c>
     </row>
@@ -3772,7 +3794,7 @@
       <c r="A5" t="s">
         <v>148</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>189</v>
       </c>
     </row>
@@ -3780,311 +3802,335 @@
       <c r="A6" t="s">
         <v>149</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>150</v>
+        <v>278</v>
       </c>
       <c r="B7" t="s">
-        <v>150</v>
+        <v>187</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B8" t="s">
-        <v>187</v>
+        <v>150</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>152</v>
-      </c>
-      <c r="B9" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="B9" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>153</v>
-      </c>
-      <c r="B10" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B10" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>154</v>
-      </c>
-      <c r="B11" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="B11" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>155</v>
-      </c>
-      <c r="B12" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B12" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>156</v>
-      </c>
-      <c r="B13" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="B13" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>157</v>
-      </c>
-      <c r="B14" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B14" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>158</v>
-      </c>
-      <c r="B15" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="B15" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>159</v>
-      </c>
-      <c r="B16" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="B16" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>160</v>
-      </c>
-      <c r="B17" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="B17" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>161</v>
-      </c>
-      <c r="B18" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="B18" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>162</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>189</v>
+        <v>161</v>
+      </c>
+      <c r="B19" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>163</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>187</v>
+        <v>162</v>
+      </c>
+      <c r="B20" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>164</v>
-      </c>
-      <c r="B21" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="B21" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>165</v>
-      </c>
-      <c r="B22" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="B22" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>165</v>
+      </c>
+      <c r="B23" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>166</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>167</v>
-      </c>
-      <c r="B25" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="B25" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>168</v>
-      </c>
-      <c r="B26" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="B26" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>169</v>
-      </c>
-      <c r="B27" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="B27" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>170</v>
-      </c>
-      <c r="B28" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="B28" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>171</v>
-      </c>
-      <c r="B29" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="B29" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>172</v>
-      </c>
-      <c r="B30" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="B30" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>173</v>
-      </c>
-      <c r="B31" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="B31" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>174</v>
-      </c>
-      <c r="B32" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B32" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>175</v>
-      </c>
-      <c r="B33" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="B33" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B34" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>176</v>
+      </c>
+      <c r="B35" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>177</v>
       </c>
-      <c r="B35" s="1" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="1" t="s">
-        <v>276</v>
-      </c>
-      <c r="B36" s="1" t="s">
+      <c r="B36" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>178</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>188</v>
+        <v>276</v>
+      </c>
+      <c r="B37" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>179</v>
-      </c>
-      <c r="B38" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="B38" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>180</v>
-      </c>
-      <c r="B39" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="B39" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>181</v>
-      </c>
-      <c r="B40" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="B40" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>182</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>187</v>
+        <v>180</v>
+      </c>
+      <c r="B41" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>183</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>188</v>
+        <v>181</v>
+      </c>
+      <c r="B42" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>184</v>
-      </c>
-      <c r="B43" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B43" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>183</v>
+      </c>
+      <c r="B44" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>184</v>
+      </c>
+      <c r="B45" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>280</v>
+      </c>
+      <c r="B46" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>275</v>
       </c>
-      <c r="B44" s="1" t="s">
+      <c r="B47" t="s">
         <v>187</v>
       </c>
     </row>
@@ -4095,294 +4141,291 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D39"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:B40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>205</v>
       </c>
       <c r="B2" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>177</v>
       </c>
       <c r="B3" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>223</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>228</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>219</v>
       </c>
       <c r="B6" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>206</v>
       </c>
       <c r="B7" t="s">
         <v>211</v>
       </c>
-      <c r="C7" s="1"/>
-    </row>
-    <row r="8" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>218</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>213</v>
       </c>
-      <c r="C8"/>
-      <c r="D8"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>207</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>221</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>220</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>222</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>215</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>214</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>227</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="16" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>276</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" t="s">
         <v>210</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
+      <c r="A17" t="s">
         <v>224</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
+      <c r="A18" t="s">
         <v>183</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
+      <c r="A19" t="s">
         <v>182</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
+      <c r="A20" t="s">
         <v>208</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
+      <c r="A21" t="s">
         <v>166</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="22" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>164</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="23" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>165</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="24" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>168</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
+      <c r="A25" t="s">
         <v>217</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B25" t="s">
         <v>213</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
+      <c r="A26" t="s">
         <v>216</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" t="s">
         <v>213</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
+      <c r="A27" t="s">
         <v>178</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
+      <c r="A28" t="s">
         <v>179</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
+      <c r="A29" t="s">
         <v>167</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B29" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
+      <c r="A30" t="s">
         <v>229</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B30" t="s">
         <v>210</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
+      <c r="A31" t="s">
         <v>230</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B31" t="s">
         <v>210</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
+      <c r="A32" t="s">
         <v>226</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B32" t="s">
         <v>210</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" s="1" t="s">
+      <c r="A33" t="s">
         <v>225</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B33" t="s">
         <v>210</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" s="1" t="s">
+      <c r="A34" t="s">
         <v>180</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B34" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="35" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="1" t="s">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>277</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B35" t="s">
         <v>211</v>
       </c>
     </row>
@@ -4406,7 +4449,7 @@
       <c r="A38" t="s">
         <v>169</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="B38" t="s">
         <v>212</v>
       </c>
     </row>
@@ -4414,12 +4457,20 @@
       <c r="A39" t="s">
         <v>184</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="B39" t="s">
         <v>212</v>
       </c>
     </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>281</v>
+      </c>
+      <c r="B40" t="s">
+        <v>212</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState ref="D2:D71">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="D2:D71">
     <sortCondition ref="D71"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>